<commit_message>
Add student import, CRUD and UI improvements
Introduce bulk student import and comprehensive student management changes: add SiswaImport class and siswa.xlsx format, enhance SiswaController with index, store, import, edit, update, toggleStatus and destroy actions (with validation and DB transactions), and integrate Maatwebsite Excel for imports. Refactor views: remove siswa/create, redesign siswa/edit, revamp siswa/index with add/import modals, status toggle, delete confirmation, DataTable init, SweetAlert2 toasts and custom file-input handling; move/import modal in mapel index. Improve MapelImport date/time parsing and uppercase tokens. Update routes to register new student endpoints and bump axios in package.json to ^1.15.0.
</commit_message>
<xml_diff>
--- a/public/assets/format_excel/mapel.xlsx
+++ b/public/assets/format_excel/mapel.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nikko\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\ujian\public\assets\format_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDEA2818-252F-4E17-854E-2B0A7C6F7D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0306DAD6-BE13-4966-83A1-76A4D9B6C96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{10FE4C57-2589-4B61-99CD-ECEA947F5EB7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{10FE4C57-2589-4B61-99CD-ECEA947F5EB7}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Mapel" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="39">
   <si>
     <t>no</t>
   </si>
@@ -119,13 +117,40 @@
     <t>TES MAPEL LPK3</t>
   </si>
   <si>
-    <t>04/13/2026</t>
-  </si>
-  <si>
-    <t>04/14/2026</t>
-  </si>
-  <si>
-    <t>04/15/2026</t>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>20/04/2026</t>
+  </si>
+  <si>
+    <t>20/04/2027</t>
+  </si>
+  <si>
+    <t>20/04/2028</t>
+  </si>
+  <si>
+    <t>20/04/2029</t>
+  </si>
+  <si>
+    <t>20/04/2030</t>
+  </si>
+  <si>
+    <t>20/04/2031</t>
+  </si>
+  <si>
+    <t>07:30</t>
+  </si>
+  <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>01:00</t>
   </si>
 </sst>
 </file>
@@ -142,14 +167,17 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -160,7 +188,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -168,45 +196,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -540,226 +537,228 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85D44184-F300-4D19-B0BE-6AB26411A8C2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49B40D24-010F-493D-8F67-7AC6EE26B7FB}">
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="69.140625" customWidth="1"/>
+    <col min="1" max="1" width="3.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="56.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="3">
-        <v>46299</v>
-      </c>
-      <c r="E2" s="4">
-        <v>0.3125</v>
-      </c>
-      <c r="F2" s="4">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="G2" s="4">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="H2" s="5">
+      <c r="D2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="1">
         <v>10</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="3">
-        <v>46330</v>
-      </c>
-      <c r="E3" s="4">
-        <v>0.3125</v>
-      </c>
-      <c r="F3" s="4">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="G3" s="4">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="H3" s="5">
+      <c r="D3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H3" s="1">
         <v>10</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="3">
-        <v>46360</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0.3125</v>
-      </c>
-      <c r="F4" s="4">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="G4" s="4">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="H4" s="5">
+      <c r="D4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="1">
         <v>10</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>1</v>
-      </c>
-      <c r="B5" s="2" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="4">
-        <v>0.3125</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="G5" s="4">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="H5" s="5">
+      <c r="D5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" s="1">
         <v>10</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>1</v>
-      </c>
-      <c r="B6" s="2" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="4">
-        <v>0.3125</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="G6" s="4">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="H6" s="5">
+      <c r="D6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H6" s="1">
         <v>10</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>1</v>
-      </c>
-      <c r="B7" s="2" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="4">
-        <v>0.3125</v>
-      </c>
-      <c r="F7" s="4">
-        <v>0.35416666666666669</v>
-      </c>
-      <c r="G7" s="4">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="H7" s="5">
+      <c r="D7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H7" s="1">
         <v>10</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" s="1" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>